<commit_message>
Jul 15 SCRA 2026
</commit_message>
<xml_diff>
--- a/scra/scra_pymt_history_from_2021.xlsx
+++ b/scra/scra_pymt_history_from_2021.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="207">
   <si>
     <t>S No</t>
   </si>
@@ -298,9 +298,6 @@
   </si>
   <si>
     <t>1st Cross Street</t>
-  </si>
-  <si>
-    <t>S Padmanabhan</t>
   </si>
   <si>
     <t>Malavika Apartment</t>
@@ -1431,13 +1428,13 @@
         <v>7</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="L1" s="24" t="s">
         <v>8</v>
@@ -1474,8 +1471,8 @@
       <c r="J2" s="18">
         <v>2500</v>
       </c>
-      <c r="K2" s="36">
-        <v>0</v>
+      <c r="K2" s="18">
+        <v>2500</v>
       </c>
       <c r="L2" s="9"/>
       <c r="M2" s="10"/>
@@ -1520,7 +1517,7 @@
         <v>7500</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="M3" s="10"/>
       <c r="N3" s="11"/>
@@ -1564,7 +1561,7 @@
         <v>2500</v>
       </c>
       <c r="L4" s="9" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="M4" s="10"/>
       <c r="N4" s="11"/>
@@ -1580,7 +1577,7 @@
         <v>73</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>41</v>
@@ -1601,8 +1598,8 @@
       <c r="J5" s="9">
         <v>10000</v>
       </c>
-      <c r="K5" s="36">
-        <v>0</v>
+      <c r="K5" s="18">
+        <v>10000</v>
       </c>
       <c r="L5" s="9"/>
       <c r="M5" s="10"/>
@@ -1616,10 +1613,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>83</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>84</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>41</v>
@@ -1658,16 +1655,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="C7" s="6" t="s">
         <v>123</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>124</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>41</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F7" s="20">
         <v>0</v>
@@ -1688,7 +1685,7 @@
         <v>0</v>
       </c>
       <c r="L7" s="49" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="M7" s="10"/>
       <c r="N7" s="11"/>
@@ -1702,7 +1699,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>22</v>
@@ -1826,10 +1823,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D11" s="7" t="s">
         <v>23</v>
@@ -1868,10 +1865,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="C12" s="6" t="s">
         <v>133</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>134</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>23</v>
@@ -1898,7 +1895,7 @@
         <v>2500</v>
       </c>
       <c r="L12" s="24" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="M12" s="10"/>
       <c r="N12" s="11"/>
@@ -1912,7 +1909,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>20</v>
@@ -1942,7 +1939,7 @@
         <v>2500</v>
       </c>
       <c r="L13" s="9" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="M13" s="10"/>
       <c r="N13" s="11"/>
@@ -1986,7 +1983,7 @@
         <v>0</v>
       </c>
       <c r="L14" s="25" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M14" s="10"/>
       <c r="N14" s="11"/>
@@ -2000,28 +1997,28 @@
         <v>14</v>
       </c>
       <c r="B15" s="52" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C15" s="52" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D15" s="48" t="s">
         <v>34</v>
       </c>
       <c r="E15" s="48" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J15" s="9">
         <v>1500</v>
@@ -2042,16 +2039,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="52" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C16" s="52" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D16" s="48" t="s">
         <v>34</v>
       </c>
       <c r="E16" s="48" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F16" s="8"/>
       <c r="G16" s="8"/>
@@ -2076,16 +2073,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="52" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C17" s="52" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D17" s="48" t="s">
         <v>34</v>
       </c>
       <c r="E17" s="48" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F17" s="8"/>
       <c r="G17" s="8"/>
@@ -2110,7 +2107,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>20</v>
@@ -2152,10 +2149,10 @@
         <v>18</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D19" s="7" t="s">
         <v>21</v>
@@ -2194,16 +2191,16 @@
         <v>19</v>
       </c>
       <c r="B20" s="52" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C20" s="52" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D20" s="48" t="s">
         <v>34</v>
       </c>
       <c r="E20" s="48" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F20" s="8"/>
       <c r="G20" s="8"/>
@@ -2252,7 +2249,7 @@
         <v>1500</v>
       </c>
       <c r="J21" s="18" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="K21" s="36">
         <v>0</v>
@@ -2300,7 +2297,7 @@
         <v>2500</v>
       </c>
       <c r="L22" s="9" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="M22" s="10"/>
       <c r="N22" s="11"/>
@@ -2314,16 +2311,16 @@
         <v>22</v>
       </c>
       <c r="B23" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C23" s="6" t="s">
         <v>101</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>102</v>
       </c>
       <c r="D23" s="7" t="s">
         <v>34</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F23" s="8">
         <v>0</v>
@@ -2356,10 +2353,10 @@
         <v>23</v>
       </c>
       <c r="B24" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C24" s="6" t="s">
         <v>104</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>105</v>
       </c>
       <c r="D24" s="7" t="s">
         <v>34</v>
@@ -2398,16 +2395,16 @@
         <v>24</v>
       </c>
       <c r="B25" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C25" s="6" t="s">
         <v>121</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>122</v>
       </c>
       <c r="D25" s="7" t="s">
         <v>34</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F25" s="8">
         <v>0</v>
@@ -2440,10 +2437,10 @@
         <v>25</v>
       </c>
       <c r="B26" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="C26" s="6" t="s">
         <v>142</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>143</v>
       </c>
       <c r="D26" s="7" t="s">
         <v>34</v>
@@ -2566,10 +2563,10 @@
         <v>28</v>
       </c>
       <c r="B29" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C29" s="6" t="s">
         <v>76</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>77</v>
       </c>
       <c r="D29" s="7" t="s">
         <v>17</v>
@@ -2608,10 +2605,10 @@
         <v>29</v>
       </c>
       <c r="B30" s="52" t="s">
+        <v>185</v>
+      </c>
+      <c r="C30" s="52" t="s">
         <v>186</v>
-      </c>
-      <c r="C30" s="52" t="s">
-        <v>187</v>
       </c>
       <c r="D30" s="48" t="s">
         <v>11</v>
@@ -2648,10 +2645,10 @@
         <v>30</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>17</v>
@@ -2678,7 +2675,7 @@
         <v>0</v>
       </c>
       <c r="L31" s="24" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="M31" s="10"/>
       <c r="N31" s="11"/>
@@ -2692,16 +2689,16 @@
         <v>31</v>
       </c>
       <c r="B32" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="C32" s="6" t="s">
         <v>113</v>
-      </c>
-      <c r="C32" s="6" t="s">
-        <v>114</v>
       </c>
       <c r="D32" s="7" t="s">
         <v>17</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F32" s="8">
         <v>0</v>
@@ -2734,16 +2731,16 @@
         <v>32</v>
       </c>
       <c r="B33" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="C33" s="6" t="s">
         <v>116</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>117</v>
       </c>
       <c r="D33" s="7" t="s">
         <v>17</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F33" s="8">
         <v>0</v>
@@ -2776,16 +2773,16 @@
         <v>33</v>
       </c>
       <c r="B34" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C34" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="D34" s="7" t="s">
         <v>17</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F34" s="8">
         <v>0</v>
@@ -2818,16 +2815,16 @@
         <v>34</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D35" s="7" t="s">
         <v>17</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F35" s="8">
         <v>0</v>
@@ -2860,16 +2857,16 @@
         <v>35</v>
       </c>
       <c r="B36" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="C36" s="6" t="s">
         <v>131</v>
-      </c>
-      <c r="C36" s="6" t="s">
-        <v>132</v>
       </c>
       <c r="D36" s="7" t="s">
         <v>17</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F36" s="8">
         <v>0</v>
@@ -2902,10 +2899,10 @@
         <v>36</v>
       </c>
       <c r="B37" s="52" t="s">
+        <v>205</v>
+      </c>
+      <c r="C37" s="52" t="s">
         <v>206</v>
-      </c>
-      <c r="C37" s="52" t="s">
-        <v>207</v>
       </c>
       <c r="D37" s="48" t="s">
         <v>23</v>
@@ -2972,7 +2969,7 @@
         <v>0</v>
       </c>
       <c r="L38" s="9" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="M38" s="10"/>
       <c r="N38" s="11"/>
@@ -3016,7 +3013,7 @@
         <v>0</v>
       </c>
       <c r="L39" s="9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="M39" s="10"/>
       <c r="N39" s="11"/>
@@ -3060,7 +3057,7 @@
         <v>0</v>
       </c>
       <c r="L40" s="9" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="M40" s="10"/>
       <c r="N40" s="11"/>
@@ -3074,7 +3071,7 @@
         <v>40</v>
       </c>
       <c r="B41" s="41" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C41" s="40"/>
       <c r="D41" s="41"/>
@@ -3100,10 +3097,10 @@
         <v>41</v>
       </c>
       <c r="B42" s="55" t="s">
+        <v>203</v>
+      </c>
+      <c r="C42" s="54" t="s">
         <v>204</v>
-      </c>
-      <c r="C42" s="54" t="s">
-        <v>205</v>
       </c>
       <c r="D42" s="55" t="s">
         <v>11</v>
@@ -3218,7 +3215,7 @@
         <v>44</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C45" s="6" t="s">
         <v>30</v>
@@ -3248,7 +3245,7 @@
         <v>0</v>
       </c>
       <c r="L45" s="9" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="M45" s="10"/>
       <c r="N45" s="11"/>
@@ -3262,10 +3259,10 @@
         <v>45</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D46" s="7" t="s">
         <v>31</v>
@@ -3304,10 +3301,10 @@
         <v>46</v>
       </c>
       <c r="B47" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="C47" s="6" t="s">
         <v>88</v>
-      </c>
-      <c r="C47" s="6" t="s">
-        <v>89</v>
       </c>
       <c r="D47" s="7" t="s">
         <v>31</v>
@@ -3346,10 +3343,10 @@
         <v>47</v>
       </c>
       <c r="B48" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="C48" s="6" t="s">
         <v>90</v>
-      </c>
-      <c r="C48" s="6" t="s">
-        <v>91</v>
       </c>
       <c r="D48" s="7" t="s">
         <v>31</v>
@@ -3388,10 +3385,10 @@
         <v>48</v>
       </c>
       <c r="B49" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C49" s="6" t="s">
         <v>95</v>
-      </c>
-      <c r="C49" s="6" t="s">
-        <v>96</v>
       </c>
       <c r="D49" s="7" t="s">
         <v>31</v>
@@ -3430,10 +3427,10 @@
         <v>49</v>
       </c>
       <c r="B50" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C50" s="6" t="s">
         <v>97</v>
-      </c>
-      <c r="C50" s="6" t="s">
-        <v>98</v>
       </c>
       <c r="D50" s="7" t="s">
         <v>31</v>
@@ -3472,7 +3469,7 @@
         <v>50</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C51" s="6" t="s">
         <v>30</v>
@@ -3514,10 +3511,10 @@
         <v>51</v>
       </c>
       <c r="B52" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="C52" s="6" t="s">
         <v>106</v>
-      </c>
-      <c r="C52" s="6" t="s">
-        <v>107</v>
       </c>
       <c r="D52" s="7" t="s">
         <v>31</v>
@@ -3556,7 +3553,7 @@
         <v>52</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C53" s="6" t="s">
         <v>30</v>
@@ -3598,10 +3595,10 @@
         <v>53</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D54" s="7" t="s">
         <v>31</v>
@@ -3640,10 +3637,10 @@
         <v>54</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D55" s="7" t="s">
         <v>31</v>
@@ -3670,7 +3667,7 @@
         <v>2500</v>
       </c>
       <c r="L55" s="24" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="M55" s="10"/>
       <c r="N55" s="11"/>
@@ -3684,10 +3681,10 @@
         <v>55</v>
       </c>
       <c r="B56" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="C56" s="6" t="s">
         <v>127</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>128</v>
       </c>
       <c r="D56" s="7" t="s">
         <v>31</v>
@@ -3714,7 +3711,7 @@
         <v>0</v>
       </c>
       <c r="L56" s="24" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="M56" s="10"/>
       <c r="N56" s="11"/>
@@ -3728,16 +3725,16 @@
         <v>56</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D57" s="7" t="s">
         <v>31</v>
       </c>
       <c r="E57" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F57" s="8">
         <v>0</v>
@@ -3770,7 +3767,7 @@
         <v>57</v>
       </c>
       <c r="B58" s="40" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C58" s="40"/>
       <c r="D58" s="41"/>
@@ -3796,7 +3793,7 @@
         <v>58</v>
       </c>
       <c r="B59" s="40" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C59" s="40"/>
       <c r="D59" s="41"/>
@@ -3822,7 +3819,7 @@
         <v>59</v>
       </c>
       <c r="B60" s="40" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C60" s="40"/>
       <c r="D60" s="41"/>
@@ -3890,16 +3887,16 @@
         <v>61</v>
       </c>
       <c r="B62" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="C62" s="6" t="s">
         <v>163</v>
-      </c>
-      <c r="C62" s="6" t="s">
-        <v>164</v>
       </c>
       <c r="D62" s="48" t="s">
         <v>58</v>
       </c>
       <c r="E62" s="48" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F62" s="16">
         <v>0</v>
@@ -4011,10 +4008,10 @@
         <v>64</v>
       </c>
       <c r="B65" s="15" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D65" s="7" t="s">
         <v>50</v>
@@ -4048,28 +4045,28 @@
         <v>65</v>
       </c>
       <c r="B66" s="54" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C66" s="54" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D66" s="55" t="s">
         <v>58</v>
       </c>
       <c r="E66" s="55" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F66" s="56" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G66" s="56" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H66" s="56" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I66" s="56" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J66" s="56"/>
       <c r="K66" s="8">
@@ -4083,10 +4080,10 @@
         <v>66</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D67" s="7" t="s">
         <v>50</v>
@@ -4120,10 +4117,10 @@
         <v>67</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D68" s="7" t="s">
         <v>50</v>
@@ -4160,7 +4157,7 @@
         <v>61</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D69" s="7" t="s">
         <v>11</v>
@@ -4224,7 +4221,7 @@
         <v>7500</v>
       </c>
       <c r="L70" s="9" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.25">
@@ -4279,7 +4276,7 @@
         <v>11</v>
       </c>
       <c r="E72" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F72" s="8">
         <v>10000</v>
@@ -4307,7 +4304,7 @@
         <v>72</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C73" s="6" t="s">
         <v>19</v>
@@ -4316,7 +4313,7 @@
         <v>11</v>
       </c>
       <c r="E73" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F73" s="8"/>
       <c r="G73" s="20"/>
@@ -4408,7 +4405,7 @@
         <v>75</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C76" s="6" t="s">
         <v>28</v>
@@ -4556,7 +4553,7 @@
         <v>79</v>
       </c>
       <c r="B80" s="40" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C80" s="40"/>
       <c r="D80" s="41"/>
@@ -4577,28 +4574,28 @@
         <v>80</v>
       </c>
       <c r="B81" s="40" t="s">
+        <v>156</v>
+      </c>
+      <c r="C81" s="40" t="s">
         <v>157</v>
       </c>
-      <c r="C81" s="40" t="s">
-        <v>158</v>
-      </c>
       <c r="D81" s="41" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E81" s="41" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F81" s="38" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G81" s="38" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H81" s="42" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I81" s="42" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J81" s="42"/>
       <c r="K81" s="36">
@@ -4612,7 +4609,7 @@
         <v>81</v>
       </c>
       <c r="B82" s="40" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C82" s="40"/>
       <c r="D82" s="41"/>
@@ -4670,10 +4667,10 @@
         <v>83</v>
       </c>
       <c r="B84" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C84" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D84" s="7" t="s">
         <v>11</v>
@@ -4696,7 +4693,7 @@
         <v>0</v>
       </c>
       <c r="L84" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="85" spans="1:12" x14ac:dyDescent="0.25">
@@ -4705,10 +4702,10 @@
         <v>84</v>
       </c>
       <c r="B85" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="C85" s="6" t="s">
         <v>80</v>
-      </c>
-      <c r="C85" s="6" t="s">
-        <v>81</v>
       </c>
       <c r="D85" s="7" t="s">
         <v>11</v>
@@ -4735,7 +4732,7 @@
         <v>2500</v>
       </c>
       <c r="L85" s="9" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="86" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -4744,10 +4741,10 @@
         <v>85</v>
       </c>
       <c r="B86" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C86" s="6" t="s">
         <v>85</v>
-      </c>
-      <c r="C86" s="6" t="s">
-        <v>86</v>
       </c>
       <c r="D86" s="7" t="s">
         <v>11</v>
@@ -4781,7 +4778,7 @@
         <v>86</v>
       </c>
       <c r="B87" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C87" s="6" t="s">
         <v>10</v>
@@ -4807,11 +4804,11 @@
       <c r="J87" s="9">
         <v>2500</v>
       </c>
-      <c r="K87" s="36">
-        <v>0</v>
+      <c r="K87" s="18">
+        <v>2500</v>
       </c>
       <c r="L87" s="9" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="88" spans="1:12" x14ac:dyDescent="0.25">
@@ -4820,10 +4817,10 @@
         <v>87</v>
       </c>
       <c r="B88" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C88" s="6" t="s">
         <v>93</v>
-      </c>
-      <c r="C88" s="6" t="s">
-        <v>94</v>
       </c>
       <c r="D88" s="7" t="s">
         <v>11</v>
@@ -4857,7 +4854,7 @@
         <v>88</v>
       </c>
       <c r="B89" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C89" s="6" t="s">
         <v>10</v>
@@ -4894,10 +4891,10 @@
         <v>89</v>
       </c>
       <c r="B90" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C90" s="6" t="s">
         <v>110</v>
-      </c>
-      <c r="C90" s="6" t="s">
-        <v>111</v>
       </c>
       <c r="D90" s="7" t="s">
         <v>11</v>
@@ -4931,10 +4928,10 @@
         <v>90</v>
       </c>
       <c r="B91" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C91" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D91" s="6" t="s">
         <v>11</v>
@@ -4966,16 +4963,16 @@
         <v>91</v>
       </c>
       <c r="B92" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="C92" s="6" t="s">
         <v>150</v>
-      </c>
-      <c r="C92" s="6" t="s">
-        <v>151</v>
       </c>
       <c r="D92" s="6" t="s">
         <v>11</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F92" s="20"/>
       <c r="G92" s="20"/>
@@ -4997,16 +4994,16 @@
         <v>92</v>
       </c>
       <c r="B93" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="C93" s="6" t="s">
         <v>147</v>
-      </c>
-      <c r="C93" s="6" t="s">
-        <v>148</v>
       </c>
       <c r="D93" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E93" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F93" s="20">
         <v>0</v>
@@ -5027,7 +5024,7 @@
         <v>1500</v>
       </c>
       <c r="L93" s="9" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="94" spans="1:12" ht="45" x14ac:dyDescent="0.25">
@@ -5039,13 +5036,13 @@
         <v>24</v>
       </c>
       <c r="C94" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D94" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E94" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F94" s="20">
         <v>0</v>
@@ -5073,16 +5070,16 @@
         <v>94</v>
       </c>
       <c r="B95" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C95" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D95" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E95" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F95" s="20">
         <v>0</v>
@@ -5110,10 +5107,10 @@
         <v>95</v>
       </c>
       <c r="B96" s="53" t="s">
+        <v>177</v>
+      </c>
+      <c r="C96" s="54" t="s">
         <v>178</v>
-      </c>
-      <c r="C96" s="54" t="s">
-        <v>179</v>
       </c>
       <c r="D96" s="55" t="s">
         <v>31</v>
@@ -5122,13 +5119,13 @@
         <v>12</v>
       </c>
       <c r="F96" s="17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G96" s="17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H96" s="17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I96" s="16">
         <v>2500</v>
@@ -5147,7 +5144,7 @@
         <v>96</v>
       </c>
       <c r="B97" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C97" s="6"/>
       <c r="D97" s="48" t="s">
@@ -5182,12 +5179,12 @@
         <v>97</v>
       </c>
       <c r="B98" s="15" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C98" s="6"/>
       <c r="D98" s="48"/>
       <c r="E98" s="48" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F98" s="17">
         <v>0</v>
@@ -5228,7 +5225,7 @@
     </row>
     <row r="101" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
       <c r="C101" s="27" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D101" s="28"/>
       <c r="E101" s="28"/>
@@ -5253,7 +5250,7 @@
     <row r="103" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
       <c r="D103" s="28"/>
       <c r="E103" s="30" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F103" s="32">
         <f>COUNTIFS(E2:E98, "House", F2:F98, "&lt;&gt;0")</f>
@@ -5277,13 +5274,13 @@
       </c>
       <c r="K103" s="32">
         <f>COUNTIFS(E2:E98, "House", K2:K98, "&lt;&gt;0")</f>
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="104" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
       <c r="D104" s="28"/>
       <c r="E104" s="30" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F104" s="32">
         <f>COUNTIFS(E2:E98, "Apartment", F2:F98, "&lt;&gt;0")</f>
@@ -5313,7 +5310,7 @@
     <row r="105" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
       <c r="D105" s="28"/>
       <c r="E105" s="30" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F105" s="32">
         <f>COUNTIFS(E2:E98, "Ind. Apartment", F2:F98, "&lt;&gt;0")</f>
@@ -5353,7 +5350,7 @@
     </row>
     <row r="108" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
       <c r="C108" s="31" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="L108" s="37"/>
     </row>
@@ -5473,7 +5470,7 @@
       </c>
       <c r="K113" s="32">
         <f>COUNTIFS(D2:D98, "1st Cross", K2:K98, "&lt;&gt;0")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="114" spans="5:11" ht="18.75" x14ac:dyDescent="0.3">
@@ -5589,7 +5586,7 @@
       </c>
       <c r="K117" s="32">
         <f>COUNTIFS(D2:D98, "Seethammal Road", K2:K98, "&lt;&gt;0")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>